<commit_message>
Updated Phase 5 scope with code quality docs, fixes, & security limitations
</commit_message>
<xml_diff>
--- a/docs/Project_Tracker.xlsx
+++ b/docs/Project_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://potbelly-my.sharepoint.com/personal/anicia_clayton_potbelly_com/Documents/Desktop/linguallearn-portfolio/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="511" documentId="8_{C9C18196-394D-4E08-AEE3-4532190AC77C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F6BD9DB-6178-47FA-B7F1-3AE5A76A76F1}"/>
+  <xr:revisionPtr revIDLastSave="967" documentId="8_{C9C18196-394D-4E08-AEE3-4532190AC77C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32AA86B7-68A8-447D-A716-53DE05E7BA25}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,6 @@
     <sheet name="📖 How to Use" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="501">
   <si>
     <t>LINGUALLEARN AI - PROJECT TRACKER</t>
   </si>
@@ -765,9 +764,6 @@
     <t>P5-T006</t>
   </si>
   <si>
-    <t>Document 5 Incident Scenarios</t>
-  </si>
-  <si>
     <t>P5-T007</t>
   </si>
   <si>
@@ -795,9 +791,6 @@
     <t>P5-T011</t>
   </si>
   <si>
-    <t>Security Audit Checklist</t>
-  </si>
-  <si>
     <t>P5-T012</t>
   </si>
   <si>
@@ -825,19 +818,10 @@
     <t>P5-T016</t>
   </si>
   <si>
-    <t>End-to-End System Test</t>
-  </si>
-  <si>
     <t>P5-T017</t>
   </si>
   <si>
-    <t>Update Portfolio with Metrics</t>
-  </si>
-  <si>
     <t>P5-T018</t>
-  </si>
-  <si>
-    <t>Phase 5 Documentation</t>
   </si>
   <si>
     <t>P5-T019</t>
@@ -1312,23 +1296,296 @@
     <t>80 (58%)</t>
   </si>
   <si>
-    <t>Phase 5 - Monitoring</t>
-  </si>
-  <si>
     <t>MLOps Engineer Portfolio</t>
   </si>
   <si>
-    <t>Delayed 4 weeks</t>
-  </si>
-  <si>
     <t>ML Integration - 100%</t>
+  </si>
+  <si>
+    <t>Phase 5 - Monitoring &amp; Security</t>
+  </si>
+  <si>
+    <t>Blcoked</t>
+  </si>
+  <si>
+    <t>Apply DB Connection Context Manager</t>
+  </si>
+  <si>
+    <t>See docs/code-quality/CONNECTION_POOL_MANAGEMENT.md</t>
+  </si>
+  <si>
+    <t>Implement Structured Error Handling</t>
+  </si>
+  <si>
+    <t>See docs/code-quality/ERROR_HANDLING_PATTERNS.md</t>
+  </si>
+  <si>
+    <t>Fix ML Model (LogisticRegression, train/test split, quality gate)</t>
+  </si>
+  <si>
+    <t>See docs/code-quality/ML_MODEL_EVALUATION.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply Terraform Security Fixes </t>
+  </si>
+  <si>
+    <t>See docs/code-quality/INFRASTRUCTURE_SECURITY_HARDENING.md</t>
+  </si>
+  <si>
+    <t>Consolidated — verify SSH removed, ALB-only ingress</t>
+  </si>
+  <si>
+    <t>Consolidated — verify scoped Secrets Manager, separate Lambda roles</t>
+  </si>
+  <si>
+    <t>S3 encryption, RDS encryption, HTTPS on ALB</t>
+  </si>
+  <si>
+    <t>6 widgets: API latency, error rates, Lambda duration, RDS connections, S3 requests, ALB metrics</t>
+  </si>
+  <si>
+    <t>4 alarms: High error rate, Lambda throttling, RDS connection spike, API latency</t>
+  </si>
+  <si>
+    <t>Email notifications for alarm triggers</t>
+  </si>
+  <si>
+    <t>Enable VPC Flow Logs</t>
+  </si>
+  <si>
+    <t>CloudWatch log group with 30-day retention</t>
+  </si>
+  <si>
+    <t>Create Multi-Stage Dockerfile</t>
+  </si>
+  <si>
+    <t>Target image size &lt;300MB, separate build/runtime stages</t>
+  </si>
+  <si>
+    <t>Create docker-compose.yml</t>
+  </si>
+  <si>
+    <t>Test Local Container Build</t>
+  </si>
+  <si>
+    <t>docker build + docker run + health check</t>
+  </si>
+  <si>
+    <t>Create ECR Repository</t>
+  </si>
+  <si>
+    <t>Push Image to ECR</t>
+  </si>
+  <si>
+    <t>Document Docker Workflow</t>
+  </si>
+  <si>
+    <r>
+      <t>docs/DOCKER.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — build, run, push commands</t>
+    </r>
+  </si>
+  <si>
+    <t>P5-T020</t>
+  </si>
+  <si>
+    <t>P5-T021</t>
+  </si>
+  <si>
+    <t>P5-T022</t>
+  </si>
+  <si>
+    <t>P5-T023</t>
+  </si>
+  <si>
+    <t>P5-T024</t>
+  </si>
+  <si>
+    <t>P5-T025</t>
+  </si>
+  <si>
+    <t>P5-T026</t>
+  </si>
+  <si>
+    <t>P5-T027</t>
+  </si>
+  <si>
+    <t>Install Mlflow</t>
+  </si>
+  <si>
+    <t>Update Training Script with MLflow Tracking</t>
+  </si>
+  <si>
+    <t>Log params, metrics, artifacts for each run</t>
+  </si>
+  <si>
+    <t>Run 5 Experiment Variations</t>
+  </si>
+  <si>
+    <t>Vary hyperparameters, compare in MLflow UI</t>
+  </si>
+  <si>
+    <t>Register Best Model</t>
+  </si>
+  <si>
+    <t>Promote to MLflow Model Registry</t>
+  </si>
+  <si>
+    <t>Document MLflow Setup</t>
+  </si>
+  <si>
+    <r>
+      <t>docs/MLFLOW_SETUP.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — setup, usage, comparison</t>
+    </r>
+  </si>
+  <si>
+    <t>Locust</t>
+  </si>
+  <si>
+    <t>5-minute test, capture latency/throughput</t>
+  </si>
+  <si>
+    <t>P5-T028</t>
+  </si>
+  <si>
+    <t>P5-T029</t>
+  </si>
+  <si>
+    <t>P5-T030</t>
+  </si>
+  <si>
+    <t>P5-T031</t>
+  </si>
+  <si>
+    <t>P5-T032</t>
+  </si>
+  <si>
+    <t>P5-T033</t>
+  </si>
+  <si>
+    <t>slowapi with tiered limits (100/min general, 20/min predictions)</t>
+  </si>
+  <si>
+    <t>Add Custom ML CloudWatch Metrics</t>
+  </si>
+  <si>
+    <t>Prediction latency, model version, recall probability distribution</t>
+  </si>
+  <si>
+    <t>Update README with Phase 5 Changes</t>
+  </si>
+  <si>
+    <t>Monitoring, Docker, MLflow sections</t>
+  </si>
+  <si>
+    <t>Create MONITORING.md</t>
+  </si>
+  <si>
+    <t>Dashboard overview, alarm thresholds, runbook reference</t>
+  </si>
+  <si>
+    <t>Final Phase 5 Verification</t>
+  </si>
+  <si>
+    <t>End-to-end test: API → Lambda → CloudWatch → Alarm</t>
+  </si>
+  <si>
+    <t>P5-T034</t>
+  </si>
+  <si>
+    <t>Phase 5</t>
+  </si>
+  <si>
+    <t>B004</t>
+  </si>
+  <si>
+    <t>B005</t>
+  </si>
+  <si>
+    <t>B006</t>
+  </si>
+  <si>
+    <t>B007</t>
+  </si>
+  <si>
+    <t>B008</t>
+  </si>
+  <si>
+    <t>B009</t>
+  </si>
+  <si>
+    <t>B010</t>
+  </si>
+  <si>
+    <t>Security review identified connection pooling that needs remediation</t>
+  </si>
+  <si>
+    <t>Security review identified  error handling that needs remediation</t>
+  </si>
+  <si>
+    <t>Security review identified  ML evaluation patterns that needs remediation</t>
+  </si>
+  <si>
+    <t>Security review identified permission issues that need remediation</t>
+  </si>
+  <si>
+    <t>Scope Addition</t>
+  </si>
+  <si>
+    <t>Added "Code Quality &amp; Security Hardening" day based on collaborative security review. Includes: context manager for DB connections, structured error handling, ML model fixes (LogisticRegression, train/test split, quality gate), Terraform security (scoped IAM, separated Lambda roles, S3 blocks, SSH removal)</t>
+  </si>
+  <si>
+    <t>Schedule Update</t>
+  </si>
+  <si>
+    <t>Day 1 now covers code quality fixes (6.25 hrs); total Phase 5 timeline adjusted to ~23 hours</t>
+  </si>
+  <si>
+    <t>Phase 6</t>
+  </si>
+  <si>
+    <t>Scope Reduction</t>
+  </si>
+  <si>
+    <t>"Refactor API code" task reduced to formatting/linting only; substantive refactoring moved to Phase 5 Day 1</t>
+  </si>
+  <si>
+    <t>Addition</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>Added SECURITY_CONSIDERATIONS.md documenting auth approach as known limitation with solutions</t>
+  </si>
+  <si>
+    <t>Added docs/code-quality folder with lessons learned: CONNECTION_POOL_MANAGEMENT.md, ERROR_HANDLING_PATTERNS.md, ML_MODEL_EVALUATION.md, INFRASTRUCTURE_SECURITY_HARDENING.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1376,11 +1633,6 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1399,6 +1651,36 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="14">
@@ -1481,7 +1763,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1528,11 +1810,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1563,7 +1856,7 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1575,25 +1868,22 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1617,6 +1907,24 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1628,29 +1936,34 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1868,10 +2181,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2160,7 +2469,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="19.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.109375" bestFit="1" customWidth="1"/>
@@ -2171,132 +2480,132 @@
     <col min="8" max="8" width="29.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:8" ht="30" customHeight="1">
+      <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="35" t="s">
-        <v>420</v>
-      </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B4" s="40" t="s">
+        <v>414</v>
+      </c>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="35" t="s">
-        <v>395</v>
-      </c>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="35"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B5" s="40" t="s">
+        <v>390</v>
+      </c>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="35" t="s">
-        <v>419</v>
-      </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B7" s="40" t="s">
+        <v>416</v>
+      </c>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="40"/>
+      <c r="H7" s="40"/>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="35" t="s">
-        <v>421</v>
-      </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B8" s="40" t="s">
+        <v>417</v>
+      </c>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="35" t="s">
-        <v>377</v>
-      </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="34" t="s">
+      <c r="B10" s="40" t="s">
+        <v>372</v>
+      </c>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
+      <c r="G10" s="40"/>
+      <c r="H10" s="40"/>
+    </row>
+    <row r="13" spans="1:8" ht="15.6" customHeight="1">
+      <c r="A13" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="40"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="40"/>
+    </row>
+    <row r="14" spans="1:8" ht="28.8" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
@@ -2322,7 +2631,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8">
       <c r="A15" s="4">
         <v>1</v>
       </c>
@@ -2350,14 +2659,14 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8">
       <c r="A16" s="4">
         <v>2</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="26" t="s">
         <v>20</v>
       </c>
       <c r="D16" s="4" t="s">
@@ -2375,17 +2684,17 @@
         <v>0</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" s="4">
         <v>3</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="28" t="s">
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
@@ -2403,17 +2712,17 @@
         <v>0</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" s="4">
         <v>4</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="28" t="s">
         <v>20</v>
       </c>
       <c r="D18" s="4" t="s">
@@ -2431,10 +2740,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="4">
         <v>5</v>
       </c>
@@ -2442,7 +2751,7 @@
         <v>35</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>36</v>
@@ -2451,7 +2760,7 @@
         <v>37</v>
       </c>
       <c r="F19" s="16">
-        <f>IFERROR(COUNTIF('Phase 5 - Monitoring'!E5:E100,"Complete")/COUNTA('Phase 5 - Monitoring'!A5:A100),0)</f>
+        <f>IFERROR(COUNTIF('Phase 5 - Monitoring'!E5:E115,"Complete")/COUNTA('Phase 5 - Monitoring'!A5:A115),0)</f>
         <v>0</v>
       </c>
       <c r="G19" s="4">
@@ -2460,7 +2769,7 @@
       </c>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8">
       <c r="A20" s="4">
         <v>6</v>
       </c>
@@ -2486,29 +2795,29 @@
       </c>
       <c r="H20" s="4"/>
     </row>
-    <row r="23" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="15.6" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8">
       <c r="A24" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B24">
         <f>COUNTA('Phase 1 - Infrastructure'!A:A)+COUNTA('Phase 2 - API &amp; Compute'!A:A)+COUNTA('Phase 3 - Multi-Modal'!A:A)+COUNTA('Phase 4 - ML Integration'!A:A)+COUNTA('Phase 5 - Monitoring'!A:A)+COUNTA('Phase 6 - CICD'!A:A)</f>
-        <v>137</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B25" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" s="1" t="s">
         <v>44</v>
       </c>
@@ -2516,7 +2825,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8">
       <c r="A27" s="1" t="s">
         <v>46</v>
       </c>
@@ -2524,18 +2833,18 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8">
       <c r="A28" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B28" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" s="8"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8">
       <c r="A30" s="1" t="s">
         <v>49</v>
       </c>
@@ -2543,15 +2852,15 @@
         <v>50</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8">
       <c r="A31" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B31" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" s="1" t="s">
         <v>52</v>
       </c>
@@ -2578,223 +2887,223 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="70" customWidth="1"/>
     <col min="3" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:6" ht="25.05" customHeight="1">
+      <c r="A1" s="42" t="s">
+        <v>323</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+    </row>
+    <row r="4" spans="1:6" ht="15.6" customHeight="1">
+      <c r="A4" s="39" t="s">
+        <v>324</v>
+      </c>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="B5" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B6" t="s">
         <v>328</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="B7" t="s">
         <v>330</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="1" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="B8" t="s">
         <v>332</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="10" spans="1:6" ht="15.6" customHeight="1">
+      <c r="A10" s="39" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="B10" s="40"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B11" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+    <row r="12" spans="1:6">
+      <c r="A12" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B12" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="34" t="s">
+    <row r="13" spans="1:6">
+      <c r="A13" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B10" s="35"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="B13" t="s">
         <v>339</v>
       </c>
-      <c r="B11" t="s">
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="1" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="B14" t="s">
         <v>341</v>
       </c>
-      <c r="B12" t="s">
+    </row>
+    <row r="16" spans="1:6" ht="15.6" customHeight="1">
+      <c r="A16" s="39" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="B16" s="40"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B17" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+    <row r="18" spans="1:6">
+      <c r="A18" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B18" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="34" t="s">
+    <row r="19" spans="1:6">
+      <c r="A19" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="B19" t="s">
         <v>348</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="1" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="B20" t="s">
         <v>350</v>
       </c>
-      <c r="B18" t="s">
+    </row>
+    <row r="22" spans="1:6" ht="15.6" customHeight="1">
+      <c r="A22" s="39" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+      <c r="B22" s="40"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B23" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
+    <row r="24" spans="1:6">
+      <c r="A24" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B24" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="34" t="s">
+    <row r="25" spans="1:6">
+      <c r="A25" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+      <c r="B25" t="s">
         <v>357</v>
       </c>
-      <c r="B23" t="s">
+    </row>
+    <row r="27" spans="1:6" ht="15.6" customHeight="1">
+      <c r="A27" s="39" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+      <c r="B27" s="40"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B28" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+    <row r="29" spans="1:6">
+      <c r="A29" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B29" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="34" t="s">
+    <row r="30" spans="1:6">
+      <c r="A30" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="B27" s="35"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+      <c r="B30" t="s">
         <v>364</v>
       </c>
-      <c r="B28" t="s">
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="1" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
+      <c r="B31" t="s">
         <v>366</v>
-      </c>
-      <c r="B29" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="B30" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="B31" t="s">
-        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -2813,7 +3122,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="8.5546875" customWidth="1"/>
@@ -2826,21 +3135,21 @@
     <col min="10" max="10" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:10" ht="25.05" customHeight="1">
+      <c r="A1" s="42" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -2848,7 +3157,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10">
       <c r="A4" s="3" t="s">
         <v>55</v>
       </c>
@@ -2880,7 +3189,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="A5" s="10" t="s">
         <v>63</v>
       </c>
@@ -2908,7 +3217,7 @@
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="A6" s="10" t="s">
         <v>68</v>
       </c>
@@ -2936,7 +3245,7 @@
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10">
       <c r="A7" s="10" t="s">
         <v>70</v>
       </c>
@@ -2964,7 +3273,7 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10">
       <c r="A8" s="10" t="s">
         <v>72</v>
       </c>
@@ -2992,7 +3301,7 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10">
       <c r="A9" s="10" t="s">
         <v>74</v>
       </c>
@@ -3022,7 +3331,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10">
       <c r="A10" s="10" t="s">
         <v>78</v>
       </c>
@@ -3050,7 +3359,7 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10">
       <c r="A11" s="10" t="s">
         <v>80</v>
       </c>
@@ -3078,7 +3387,7 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10">
       <c r="A12" s="10" t="s">
         <v>82</v>
       </c>
@@ -3108,7 +3417,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10">
       <c r="A13" s="10" t="s">
         <v>86</v>
       </c>
@@ -3136,7 +3445,7 @@
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10">
       <c r="A14" s="10" t="s">
         <v>89</v>
       </c>
@@ -3164,7 +3473,7 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10">
       <c r="A15" s="10" t="s">
         <v>91</v>
       </c>
@@ -3192,7 +3501,7 @@
       <c r="I15" s="10"/>
       <c r="J15" s="10"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10">
       <c r="A16" s="10" t="s">
         <v>95</v>
       </c>
@@ -3220,7 +3529,7 @@
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10">
       <c r="A17" s="10" t="s">
         <v>97</v>
       </c>
@@ -3248,7 +3557,7 @@
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10">
       <c r="A18" s="10" t="s">
         <v>99</v>
       </c>
@@ -3309,7 +3618,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
@@ -3322,29 +3631,29 @@
     <col min="10" max="10" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:10" ht="25.05" customHeight="1">
+      <c r="A1" s="42" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="26" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B2" s="25" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="3" t="s">
         <v>55</v>
       </c>
@@ -3376,7 +3685,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="A5" s="10" t="s">
         <v>103</v>
       </c>
@@ -3404,7 +3713,7 @@
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="A6" s="10" t="s">
         <v>105</v>
       </c>
@@ -3432,7 +3741,7 @@
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10">
       <c r="A7" s="10" t="s">
         <v>107</v>
       </c>
@@ -3460,7 +3769,7 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10">
       <c r="A8" s="10" t="s">
         <v>109</v>
       </c>
@@ -3492,7 +3801,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10">
       <c r="A9" s="10" t="s">
         <v>113</v>
       </c>
@@ -3524,7 +3833,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10">
       <c r="A10" s="10" t="s">
         <v>117</v>
       </c>
@@ -3552,7 +3861,7 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10">
       <c r="A11" s="10" t="s">
         <v>119</v>
       </c>
@@ -3580,7 +3889,7 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10">
       <c r="A12" s="10" t="s">
         <v>121</v>
       </c>
@@ -3608,7 +3917,7 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10">
       <c r="A13" s="10" t="s">
         <v>123</v>
       </c>
@@ -3636,7 +3945,7 @@
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10">
       <c r="A14" s="10" t="s">
         <v>125</v>
       </c>
@@ -3664,7 +3973,7 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10">
       <c r="A15" s="10" t="s">
         <v>127</v>
       </c>
@@ -3692,7 +4001,7 @@
       <c r="I15" s="10"/>
       <c r="J15" s="10"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10">
       <c r="A16" s="10" t="s">
         <v>129</v>
       </c>
@@ -3720,7 +4029,7 @@
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10">
       <c r="A17" s="10" t="s">
         <v>131</v>
       </c>
@@ -3748,7 +4057,7 @@
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10">
       <c r="A18" s="10" t="s">
         <v>133</v>
       </c>
@@ -3776,7 +4085,7 @@
       <c r="I18" s="10"/>
       <c r="J18" s="10"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10">
       <c r="A19" s="10" t="s">
         <v>135</v>
       </c>
@@ -3804,7 +4113,7 @@
       <c r="I19" s="10"/>
       <c r="J19" s="10"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10">
       <c r="A20" s="10" t="s">
         <v>137</v>
       </c>
@@ -3832,7 +4141,7 @@
       <c r="I20" s="10"/>
       <c r="J20" s="10"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10">
       <c r="A21" s="10" t="s">
         <v>139</v>
       </c>
@@ -3860,7 +4169,7 @@
       <c r="I21" s="10"/>
       <c r="J21" s="10"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10">
       <c r="A22" s="10" t="s">
         <v>141</v>
       </c>
@@ -3888,7 +4197,7 @@
       <c r="I22" s="10"/>
       <c r="J22" s="10"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10">
       <c r="A23" s="10" t="s">
         <v>143</v>
       </c>
@@ -3916,7 +4225,7 @@
       <c r="I23" s="10"/>
       <c r="J23" s="10"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10">
       <c r="A24" s="10" t="s">
         <v>145</v>
       </c>
@@ -3944,7 +4253,7 @@
       <c r="I24" s="10"/>
       <c r="J24" s="10"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10">
       <c r="A25" s="10" t="s">
         <v>147</v>
       </c>
@@ -4005,7 +4314,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="8.44140625" customWidth="1"/>
@@ -4018,29 +4327,29 @@
     <col min="10" max="10" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:10" ht="25.05" customHeight="1">
+      <c r="A1" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B2" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="3" t="s">
         <v>55</v>
       </c>
@@ -4072,7 +4381,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="A5" s="10" t="s">
         <v>150</v>
       </c>
@@ -4100,7 +4409,7 @@
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="A6" s="10" t="s">
         <v>152</v>
       </c>
@@ -4128,7 +4437,7 @@
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10">
       <c r="A7" s="10" t="s">
         <v>154</v>
       </c>
@@ -4156,7 +4465,7 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10">
       <c r="A8" s="10" t="s">
         <v>156</v>
       </c>
@@ -4184,7 +4493,7 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10">
       <c r="A9" s="10" t="s">
         <v>158</v>
       </c>
@@ -4212,7 +4521,7 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10">
       <c r="A10" s="10" t="s">
         <v>160</v>
       </c>
@@ -4240,7 +4549,7 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10">
       <c r="A11" s="10" t="s">
         <v>162</v>
       </c>
@@ -4267,10 +4576,10 @@
       </c>
       <c r="I11" s="10"/>
       <c r="J11" s="10" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" s="10" t="s">
         <v>164</v>
       </c>
@@ -4298,7 +4607,7 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10">
       <c r="A13" s="10" t="s">
         <v>166</v>
       </c>
@@ -4326,7 +4635,7 @@
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10">
       <c r="A14" s="10" t="s">
         <v>168</v>
       </c>
@@ -4334,7 +4643,7 @@
         <v>83</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>66</v>
@@ -4354,7 +4663,7 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10">
       <c r="A15" s="10" t="s">
         <v>170</v>
       </c>
@@ -4362,7 +4671,7 @@
         <v>83</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>66</v>
@@ -4382,7 +4691,7 @@
       <c r="I15" s="10"/>
       <c r="J15" s="10"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10">
       <c r="A16" s="10" t="s">
         <v>172</v>
       </c>
@@ -4390,7 +4699,7 @@
         <v>83</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>66</v>
@@ -4410,7 +4719,7 @@
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10">
       <c r="A17" s="10" t="s">
         <v>174</v>
       </c>
@@ -4418,7 +4727,7 @@
         <v>83</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>66</v>
@@ -4438,7 +4747,7 @@
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10">
       <c r="A18" s="10" t="s">
         <v>176</v>
       </c>
@@ -4446,7 +4755,7 @@
         <v>83</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>66</v>
@@ -4466,7 +4775,7 @@
       <c r="I18" s="10"/>
       <c r="J18" s="10"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10">
       <c r="A19" s="10" t="s">
         <v>178</v>
       </c>
@@ -4492,13 +4801,13 @@
         <v>2.5</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
       <c r="A20" s="10" t="s">
         <v>180</v>
       </c>
@@ -4526,7 +4835,7 @@
       <c r="I20" s="10"/>
       <c r="J20" s="10"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10">
       <c r="A21" s="10" t="s">
         <v>182</v>
       </c>
@@ -4554,7 +4863,7 @@
       <c r="I21" s="10"/>
       <c r="J21" s="10"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10">
       <c r="A22" s="10" t="s">
         <v>184</v>
       </c>
@@ -4581,10 +4890,10 @@
       </c>
       <c r="I22" s="10"/>
       <c r="J22" s="10" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10">
       <c r="A23" s="10" t="s">
         <v>186</v>
       </c>
@@ -4611,10 +4920,10 @@
       </c>
       <c r="I23" s="10"/>
       <c r="J23" s="10" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10">
       <c r="A24" s="10" t="s">
         <v>188</v>
       </c>
@@ -4641,12 +4950,12 @@
       </c>
       <c r="I24" s="10"/>
       <c r="J24" s="10" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10">
       <c r="A25" s="10" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>92</v>
@@ -4672,9 +4981,9 @@
       <c r="I25" s="10"/>
       <c r="J25" s="10"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10">
       <c r="A26" s="10" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>92</v>
@@ -4700,9 +5009,9 @@
       <c r="I26" s="10"/>
       <c r="J26" s="10"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10">
       <c r="A27" s="10" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>92</v>
@@ -4728,9 +5037,9 @@
       <c r="I27" s="10"/>
       <c r="J27" s="10"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10">
       <c r="A28" s="10" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>92</v>
@@ -4756,9 +5065,9 @@
       <c r="I28" s="10"/>
       <c r="J28" s="10"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10">
       <c r="A29" s="10" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>92</v>
@@ -4817,7 +5126,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="9.77734375" customWidth="1"/>
@@ -4830,29 +5139,29 @@
     <col min="10" max="10" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:10" ht="25.05" customHeight="1">
+      <c r="A1" s="42" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B2" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="3" t="s">
         <v>55</v>
       </c>
@@ -4884,7 +5193,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="A5" s="10" t="s">
         <v>191</v>
       </c>
@@ -4912,7 +5221,7 @@
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="A6" s="10" t="s">
         <v>193</v>
       </c>
@@ -4940,7 +5249,7 @@
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10">
       <c r="A7" s="10" t="s">
         <v>195</v>
       </c>
@@ -4968,7 +5277,7 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10">
       <c r="A8" s="10" t="s">
         <v>197</v>
       </c>
@@ -4996,7 +5305,7 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10">
       <c r="A9" s="10" t="s">
         <v>199</v>
       </c>
@@ -5024,7 +5333,7 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10">
       <c r="A10" s="10" t="s">
         <v>201</v>
       </c>
@@ -5052,7 +5361,7 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10">
       <c r="A11" s="10" t="s">
         <v>203</v>
       </c>
@@ -5080,7 +5389,7 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10">
       <c r="A12" s="10" t="s">
         <v>205</v>
       </c>
@@ -5106,13 +5415,13 @@
         <v>4</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" s="10" t="s">
         <v>207</v>
       </c>
@@ -5140,7 +5449,7 @@
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10">
       <c r="A14" s="10" t="s">
         <v>209</v>
       </c>
@@ -5168,7 +5477,7 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10">
       <c r="A15" s="10" t="s">
         <v>211</v>
       </c>
@@ -5195,10 +5504,10 @@
       </c>
       <c r="I15" s="10"/>
       <c r="J15" s="10" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
       <c r="A16" s="10" t="s">
         <v>213</v>
       </c>
@@ -5224,13 +5533,13 @@
         <v>2</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="J16" s="10" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
       <c r="A17" s="10" t="s">
         <v>215</v>
       </c>
@@ -5238,7 +5547,7 @@
         <v>87</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>66</v>
@@ -5258,7 +5567,7 @@
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10">
       <c r="A18" s="10" t="s">
         <v>216</v>
       </c>
@@ -5266,7 +5575,7 @@
         <v>87</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>66</v>
@@ -5286,7 +5595,7 @@
       <c r="I18" s="10"/>
       <c r="J18" s="10"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10">
       <c r="A19" s="10" t="s">
         <v>217</v>
       </c>
@@ -5294,7 +5603,7 @@
         <v>87</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>66</v>
@@ -5312,11 +5621,11 @@
         <v>2.5</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="J19" s="10"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10">
       <c r="A20" s="10" t="s">
         <v>218</v>
       </c>
@@ -5343,10 +5652,10 @@
       </c>
       <c r="I20" s="10"/>
       <c r="J20" s="10" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
       <c r="A21" s="10" t="s">
         <v>220</v>
       </c>
@@ -5373,10 +5682,10 @@
       </c>
       <c r="I21" s="10"/>
       <c r="J21" s="10" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
       <c r="A22" s="10" t="s">
         <v>222</v>
       </c>
@@ -5404,7 +5713,7 @@
       <c r="I22" s="10"/>
       <c r="J22" s="10"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10">
       <c r="A23" s="10" t="s">
         <v>224</v>
       </c>
@@ -5432,7 +5741,7 @@
       <c r="I23" s="10"/>
       <c r="J23" s="10"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10">
       <c r="A24" s="10" t="s">
         <v>226</v>
       </c>
@@ -5493,43 +5802,43 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J38"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="3" max="3" width="59.88671875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="25" customWidth="1"/>
-    <col min="10" max="10" width="35" customWidth="1"/>
+    <col min="10" max="10" width="80.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:10" ht="25.05" customHeight="1">
+      <c r="A1" s="42" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="30" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B2" s="29" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="3" t="s">
         <v>55</v>
       </c>
@@ -5561,7 +5870,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="A5" s="10" t="s">
         <v>229</v>
       </c>
@@ -5569,7 +5878,7 @@
         <v>64</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>230</v>
+        <v>418</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>66</v>
@@ -5581,15 +5890,17 @@
         <v>67</v>
       </c>
       <c r="G5" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" s="10">
         <v>0</v>
       </c>
       <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J5" s="14" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" s="10" t="s">
         <v>231</v>
       </c>
@@ -5597,7 +5908,7 @@
         <v>64</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>232</v>
+        <v>420</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>66</v>
@@ -5615,9 +5926,11 @@
         <v>0</v>
       </c>
       <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J6" s="14" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" s="10" t="s">
         <v>233</v>
       </c>
@@ -5625,7 +5938,7 @@
         <v>64</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>234</v>
+        <v>422</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>66</v>
@@ -5637,15 +5950,17 @@
         <v>67</v>
       </c>
       <c r="G7" s="10">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="H7" s="10">
         <v>0</v>
       </c>
       <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J7" s="14" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" s="10" t="s">
         <v>235</v>
       </c>
@@ -5653,7 +5968,7 @@
         <v>64</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>236</v>
+        <v>424</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>66</v>
@@ -5661,8 +5976,8 @@
       <c r="E8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>94</v>
+      <c r="F8" s="11" t="s">
+        <v>67</v>
       </c>
       <c r="G8" s="10">
         <v>1</v>
@@ -5671,17 +5986,19 @@
         <v>0</v>
       </c>
       <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J8" s="14" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
       <c r="A9" s="10" t="s">
         <v>237</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>66</v>
@@ -5689,27 +6006,29 @@
       <c r="E9" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="11" t="s">
-        <v>67</v>
+      <c r="F9" s="48" t="s">
+        <v>94</v>
       </c>
       <c r="G9" s="10">
-        <v>3</v>
+        <v>0.25</v>
       </c>
       <c r="H9" s="10">
         <v>0</v>
       </c>
       <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J9" s="10" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
       <c r="A10" s="10" t="s">
         <v>239</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>240</v>
+        <v>64</v>
+      </c>
+      <c r="C10" t="s">
+        <v>252</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>66</v>
@@ -5717,27 +6036,29 @@
       <c r="E10" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="11" t="s">
-        <v>67</v>
+      <c r="F10" s="48" t="s">
+        <v>94</v>
       </c>
       <c r="G10" s="10">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="H10" s="10">
         <v>0</v>
       </c>
       <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J10" s="10" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>242</v>
+        <v>64</v>
+      </c>
+      <c r="C11" s="44" t="s">
+        <v>254</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>66</v>
@@ -5745,27 +6066,29 @@
       <c r="E11" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="48" t="s">
         <v>94</v>
       </c>
       <c r="G11" s="10">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="H11" s="10">
         <v>0</v>
       </c>
       <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J11" s="45" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" s="10" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>66</v>
@@ -5777,23 +6100,25 @@
         <v>67</v>
       </c>
       <c r="G12" s="10">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H12" s="10">
         <v>0</v>
       </c>
       <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J12" s="10" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" s="10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>66</v>
@@ -5805,23 +6130,25 @@
         <v>67</v>
       </c>
       <c r="G13" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="10">
         <v>0</v>
       </c>
       <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J13" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
       <c r="A14" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>66</v>
@@ -5829,27 +6156,29 @@
       <c r="E14" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>94</v>
+      <c r="F14" s="11" t="s">
+        <v>67</v>
       </c>
       <c r="G14" s="10">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H14" s="10">
         <v>0</v>
       </c>
       <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J14" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
       <c r="A15" s="10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>250</v>
+        <v>432</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>66</v>
@@ -5857,27 +6186,29 @@
       <c r="E15" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F15" s="11" t="s">
-        <v>67</v>
+      <c r="F15" s="48" t="s">
+        <v>94</v>
       </c>
       <c r="G15" s="10">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="H15" s="10">
         <v>0</v>
       </c>
       <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J15" s="45" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
       <c r="A16" s="10" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>66</v>
@@ -5885,8 +6216,8 @@
       <c r="E16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="11" t="s">
-        <v>67</v>
+      <c r="F16" s="4" t="s">
+        <v>94</v>
       </c>
       <c r="G16" s="10">
         <v>1</v>
@@ -5897,15 +6228,15 @@
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10">
       <c r="A17" s="10" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>254</v>
+        <v>238</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>66</v>
@@ -5913,27 +6244,27 @@
       <c r="E17" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="11" t="s">
-        <v>67</v>
+      <c r="F17" s="48" t="s">
+        <v>94</v>
       </c>
       <c r="G17" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H17" s="10">
         <v>0</v>
       </c>
       <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="10" t="s">
-        <v>255</v>
+      <c r="J17" s="45"/>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" s="14" t="s">
+        <v>253</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>256</v>
+        <v>434</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>66</v>
@@ -5945,23 +6276,25 @@
         <v>67</v>
       </c>
       <c r="G18" s="10">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="H18" s="10">
         <v>0</v>
       </c>
       <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="10" t="s">
-        <v>257</v>
+      <c r="J18" s="10" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" s="14" t="s">
+        <v>255</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>258</v>
+        <v>436</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>66</v>
@@ -5973,7 +6306,7 @@
         <v>94</v>
       </c>
       <c r="G19" s="10">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H19" s="10">
         <v>0</v>
@@ -5981,15 +6314,15 @@
       <c r="I19" s="10"/>
       <c r="J19" s="10"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="10" t="s">
-        <v>259</v>
+    <row r="20" spans="1:10">
+      <c r="A20" s="14" t="s">
+        <v>257</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>260</v>
+        <v>437</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>66</v>
@@ -6001,23 +6334,25 @@
         <v>67</v>
       </c>
       <c r="G20" s="10">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="H20" s="10">
         <v>0</v>
       </c>
       <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="10" t="s">
-        <v>261</v>
+      <c r="J20" s="10" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" s="14" t="s">
+        <v>258</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>262</v>
+        <v>439</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>66</v>
@@ -6025,11 +6360,11 @@
       <c r="E21" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="11" t="s">
-        <v>67</v>
+      <c r="F21" s="48" t="s">
+        <v>94</v>
       </c>
       <c r="G21" s="10">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="H21" s="10">
         <v>0</v>
@@ -6037,15 +6372,15 @@
       <c r="I21" s="10"/>
       <c r="J21" s="10"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
-        <v>263</v>
+    <row r="22" spans="1:10">
+      <c r="A22" s="14" t="s">
+        <v>259</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>264</v>
+        <v>440</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>66</v>
@@ -6053,11 +6388,11 @@
       <c r="E22" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F22" s="11" t="s">
-        <v>67</v>
+      <c r="F22" s="4" t="s">
+        <v>94</v>
       </c>
       <c r="G22" s="10">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H22" s="10">
         <v>0</v>
@@ -6065,15 +6400,15 @@
       <c r="I22" s="10"/>
       <c r="J22" s="10"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="10" t="s">
-        <v>265</v>
+    <row r="23" spans="1:10">
+      <c r="A23" s="14" t="s">
+        <v>260</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>266</v>
+        <v>441</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>66</v>
@@ -6081,23 +6416,465 @@
       <c r="E23" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="48" t="s">
         <v>101</v>
       </c>
       <c r="G23" s="10">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H23" s="10">
         <v>0</v>
       </c>
       <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
+      <c r="J23" s="46" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" s="14" t="s">
+        <v>443</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G24" s="10">
+        <v>1</v>
+      </c>
+      <c r="H24" s="10">
+        <v>0</v>
+      </c>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" s="14" t="s">
+        <v>444</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>452</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G25" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="H25" s="10">
+        <v>0</v>
+      </c>
+      <c r="I25" s="10"/>
+      <c r="J25" s="45" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="14" t="s">
+        <v>445</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>454</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F26" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="G26" s="10">
+        <v>1</v>
+      </c>
+      <c r="H26" s="10">
+        <v>0</v>
+      </c>
+      <c r="I26" s="10"/>
+      <c r="J26" s="45" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="14" t="s">
+        <v>446</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27" s="45" t="s">
+        <v>456</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F27" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="G27" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="H27" s="10">
+        <v>0</v>
+      </c>
+      <c r="I27" s="10"/>
+      <c r="J27" s="45" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" s="14" t="s">
+        <v>447</v>
+      </c>
+      <c r="B28" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" s="45" t="s">
+        <v>458</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F28" s="48" t="s">
+        <v>101</v>
+      </c>
+      <c r="G28" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="H28" s="10">
+        <v>0</v>
+      </c>
+      <c r="I28" s="10"/>
+      <c r="J28" s="46" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" s="14" t="s">
+        <v>448</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="45" t="s">
+        <v>241</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F29" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="G29" s="10">
+        <v>0.25</v>
+      </c>
+      <c r="H29" s="10">
+        <v>0</v>
+      </c>
+      <c r="I29" s="10"/>
+      <c r="J29" s="47" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" s="14" t="s">
+        <v>449</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" s="45" t="s">
+        <v>243</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F30" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="G30" s="10">
+        <v>1</v>
+      </c>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="47"/>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" s="14" t="s">
+        <v>450</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C31" s="45" t="s">
+        <v>245</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F31" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="G31" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="H31" s="10">
+        <v>0</v>
+      </c>
+      <c r="I31" s="10"/>
+      <c r="J31" s="45" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="14" t="s">
+        <v>462</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C32" s="45" t="s">
+        <v>247</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F32" s="48" t="s">
+        <v>101</v>
+      </c>
+      <c r="G32" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="H32" s="10">
+        <v>0</v>
+      </c>
+      <c r="I32" s="10"/>
+      <c r="J32" s="45"/>
+    </row>
+    <row r="33" spans="1:10">
+      <c r="A33" s="14" t="s">
+        <v>463</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F33" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="G33" s="10">
+        <v>1</v>
+      </c>
+      <c r="H33" s="10">
+        <v>0</v>
+      </c>
+      <c r="I33" s="10"/>
+      <c r="J33" s="14" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10">
+      <c r="A34" s="14" t="s">
+        <v>464</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>469</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F34" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="G34" s="10">
+        <v>1</v>
+      </c>
+      <c r="H34" s="10">
+        <v>0</v>
+      </c>
+      <c r="I34" s="10"/>
+      <c r="J34" s="14" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
+      <c r="A35" s="14" t="s">
+        <v>465</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C35" s="45" t="s">
+        <v>471</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F35" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="G35" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="H35" s="10">
+        <v>0</v>
+      </c>
+      <c r="I35" s="10"/>
+      <c r="J35" s="14" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10">
+      <c r="A36" s="14" t="s">
+        <v>466</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C36" s="45" t="s">
+        <v>473</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F36" s="48" t="s">
+        <v>101</v>
+      </c>
+      <c r="G36" s="10">
+        <v>1</v>
+      </c>
+      <c r="H36" s="10">
+        <v>0</v>
+      </c>
+      <c r="I36" s="10"/>
+      <c r="J36" s="45" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10">
+      <c r="A37" s="14" t="s">
+        <v>467</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C37" t="s">
+        <v>475</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G37" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="H37" s="10">
+        <v>0</v>
+      </c>
+      <c r="I37" s="10"/>
+      <c r="J37" s="45" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10">
+      <c r="A38" s="14" t="s">
+        <v>477</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G38" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="H38" s="10">
+        <v>0</v>
+      </c>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E100">
+  <conditionalFormatting sqref="E5:E115">
     <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"Complete"</formula>
     </cfRule>
@@ -6112,10 +6889,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" errorTitle="Invalid Entry" error="Invalid status" sqref="E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24" xr:uid="{00000000-0002-0000-0500-000000000000}">
+    <dataValidation type="list" errorTitle="Invalid Entry" error="Invalid status" sqref="E5:E12 E13 E14:E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26:E32 E33 E34 E35 E36:E37 E38 E39" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>"Not Started,In Progress,Complete,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorTitle="Invalid Entry" error="Invalid priority" sqref="F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24" xr:uid="{00000000-0002-0000-0500-000001000000}">
+    <dataValidation type="list" errorTitle="Invalid Entry" error="Invalid priority" sqref="F5:F12 F13 F14:F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26:F32 F33 F34 F35 F36:F37 F38 F39" xr:uid="{00000000-0002-0000-0500-000001000000}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6126,7 +6903,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:J24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -6139,21 +6916,21 @@
     <col min="10" max="10" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
-        <v>267</v>
-      </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="25.05" customHeight="1">
+      <c r="A1" s="42" t="s">
+        <v>262</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -6161,7 +6938,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10">
       <c r="A4" s="3" t="s">
         <v>55</v>
       </c>
@@ -6193,15 +6970,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="A5" s="10" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>64</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>66</v>
@@ -6221,15 +6998,15 @@
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="A6" s="10" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>64</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>66</v>
@@ -6249,15 +7026,15 @@
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10">
       <c r="A7" s="10" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>64</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>66</v>
@@ -6277,15 +7054,15 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10">
       <c r="A8" s="10" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>64</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>66</v>
@@ -6305,15 +7082,15 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10">
       <c r="A9" s="10" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>75</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>66</v>
@@ -6333,15 +7110,15 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10">
       <c r="A10" s="10" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>66</v>
@@ -6361,15 +7138,15 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10">
       <c r="A11" s="10" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>75</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>66</v>
@@ -6389,15 +7166,15 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10">
       <c r="A12" s="10" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>83</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>66</v>
@@ -6417,15 +7194,15 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10">
       <c r="A13" s="10" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>83</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>66</v>
@@ -6445,15 +7222,15 @@
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10">
       <c r="A14" s="10" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>83</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>66</v>
@@ -6473,15 +7250,15 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10">
       <c r="A15" s="10" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>83</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>66</v>
@@ -6501,15 +7278,15 @@
       <c r="I15" s="10"/>
       <c r="J15" s="10"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10">
       <c r="A16" s="10" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>87</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>66</v>
@@ -6529,15 +7306,15 @@
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10">
       <c r="A17" s="10" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>87</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>66</v>
@@ -6557,15 +7334,15 @@
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10">
       <c r="A18" s="10" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>87</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>66</v>
@@ -6585,15 +7362,15 @@
       <c r="I18" s="10"/>
       <c r="J18" s="10"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10">
       <c r="A19" s="10" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>87</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>66</v>
@@ -6613,15 +7390,15 @@
       <c r="I19" s="10"/>
       <c r="J19" s="10"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10">
       <c r="A20" s="10" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>92</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>66</v>
@@ -6641,15 +7418,15 @@
       <c r="I20" s="10"/>
       <c r="J20" s="10"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10">
       <c r="A21" s="10" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>92</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>66</v>
@@ -6669,15 +7446,15 @@
       <c r="I21" s="10"/>
       <c r="J21" s="10"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10">
       <c r="A22" s="10" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>92</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>66</v>
@@ -6697,15 +7474,15 @@
       <c r="I22" s="10"/>
       <c r="J22" s="10"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10">
       <c r="A23" s="10" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>92</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>66</v>
@@ -6725,15 +7502,15 @@
       <c r="I23" s="10"/>
       <c r="J23" s="10"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10">
       <c r="A24" s="10" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>92</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>66</v>
@@ -6785,8 +7562,8 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6795,26 +7572,26 @@
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="55" customWidth="1"/>
+    <col min="8" max="8" width="63.6640625" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
-        <v>308</v>
-      </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="25.05" customHeight="1">
+      <c r="A1" s="43" t="s">
+        <v>303</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" s="3" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>11</v>
@@ -6826,7 +7603,7 @@
         <v>12</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>13</v>
@@ -6835,98 +7612,287 @@
         <v>58</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="79.95" customHeight="1">
       <c r="A4" s="17" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>109</v>
       </c>
       <c r="D4" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="E4" s="50" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="I4" s="18">
+        <v>45974</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="33" customFormat="1" ht="69">
+      <c r="A5" s="19" t="s">
+        <v>312</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>309</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>313</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>314</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="20" t="s">
         <v>315</v>
       </c>
-      <c r="E4" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>319</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="H4" s="17" t="s">
-        <v>316</v>
-      </c>
-      <c r="I4" s="19">
-        <v>45974</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" s="40" customFormat="1" ht="69" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
-        <v>317</v>
-      </c>
-      <c r="B5" s="20" t="s">
+      <c r="I5" s="21">
+        <v>45975</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="41.4">
+      <c r="A6" s="34" t="s">
+        <v>409</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>400</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>217</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>408</v>
+      </c>
+      <c r="E6" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="34" t="s">
         <v>314</v>
       </c>
-      <c r="C5" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>318</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="F5" s="20" t="s">
-        <v>319</v>
-      </c>
-      <c r="G5" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="21" t="s">
-        <v>320</v>
-      </c>
-      <c r="I5" s="22">
-        <v>45975</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="41" t="s">
-        <v>414</v>
-      </c>
-      <c r="B6" s="41" t="s">
-        <v>405</v>
-      </c>
-      <c r="C6" s="41" t="s">
-        <v>217</v>
-      </c>
-      <c r="D6" s="41" t="s">
-        <v>413</v>
-      </c>
-      <c r="E6" s="44" t="s">
-        <v>94</v>
-      </c>
-      <c r="F6" s="41" t="s">
-        <v>319</v>
-      </c>
-      <c r="G6" s="41" t="s">
-        <v>66</v>
-      </c>
-      <c r="H6" s="43" t="s">
-        <v>415</v>
-      </c>
-      <c r="I6" s="42">
+      <c r="G6" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="H6" s="36" t="s">
+        <v>410</v>
+      </c>
+      <c r="I6" s="35">
         <v>46017</v>
       </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="45" t="s">
+        <v>479</v>
+      </c>
+      <c r="B7" s="45" t="s">
+        <v>478</v>
+      </c>
+      <c r="C7" s="45" t="s">
+        <v>229</v>
+      </c>
+      <c r="D7" s="51" t="s">
+        <v>486</v>
+      </c>
+      <c r="E7" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="45" t="s">
+        <v>389</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>66</v>
+      </c>
+      <c r="H7" s="45" t="s">
+        <v>419</v>
+      </c>
+      <c r="I7" s="45"/>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="45" t="s">
+        <v>480</v>
+      </c>
+      <c r="B8" s="45" t="s">
+        <v>478</v>
+      </c>
+      <c r="C8" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D8" s="51" t="s">
+        <v>487</v>
+      </c>
+      <c r="E8" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="F8" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="45" t="s">
+        <v>66</v>
+      </c>
+      <c r="H8" s="45" t="s">
+        <v>421</v>
+      </c>
+      <c r="I8" s="45"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="45" t="s">
+        <v>481</v>
+      </c>
+      <c r="B9" s="45" t="s">
+        <v>478</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>233</v>
+      </c>
+      <c r="D9" s="51" t="s">
+        <v>488</v>
+      </c>
+      <c r="E9" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="45" t="s">
+        <v>66</v>
+      </c>
+      <c r="H9" s="45" t="s">
+        <v>423</v>
+      </c>
+      <c r="I9" s="45"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="45" t="s">
+        <v>482</v>
+      </c>
+      <c r="B10" s="45" t="s">
+        <v>478</v>
+      </c>
+      <c r="C10" s="45" t="s">
+        <v>235</v>
+      </c>
+      <c r="D10" s="51" t="s">
+        <v>489</v>
+      </c>
+      <c r="E10" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="45" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="45" t="s">
+        <v>425</v>
+      </c>
+      <c r="I10" s="45"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="45" t="s">
+        <v>483</v>
+      </c>
+      <c r="B11" s="45" t="s">
+        <v>478</v>
+      </c>
+      <c r="C11" s="45" t="s">
+        <v>237</v>
+      </c>
+      <c r="D11" s="51" t="s">
+        <v>489</v>
+      </c>
+      <c r="E11" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="45" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11" s="45" t="s">
+        <v>425</v>
+      </c>
+      <c r="I11" s="45"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="45" t="s">
+        <v>484</v>
+      </c>
+      <c r="B12" s="45" t="s">
+        <v>478</v>
+      </c>
+      <c r="C12" s="45" t="s">
+        <v>239</v>
+      </c>
+      <c r="D12" s="51" t="s">
+        <v>489</v>
+      </c>
+      <c r="E12" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="45" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" s="45" t="s">
+        <v>425</v>
+      </c>
+      <c r="I12" s="45"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="45" t="s">
+        <v>485</v>
+      </c>
+      <c r="B13" s="45" t="s">
+        <v>478</v>
+      </c>
+      <c r="C13" s="45" t="s">
+        <v>240</v>
+      </c>
+      <c r="D13" s="51" t="s">
+        <v>489</v>
+      </c>
+      <c r="E13" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="F13" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="45" t="s">
+        <v>66</v>
+      </c>
+      <c r="H13" s="45" t="s">
+        <v>425</v>
+      </c>
+      <c r="I13" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6939,185 +7905,285 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="1" max="1" width="15" style="54" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="60" customWidth="1"/>
+    <col min="5" max="5" width="141.109375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
-        <v>321</v>
-      </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>322</v>
+    <row r="1" spans="1:6" ht="25.05" customHeight="1">
+      <c r="A1" s="42" t="s">
+        <v>316</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="53" t="s">
+        <v>317</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>12</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="24">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="23">
         <v>45967</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>66</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="25">
+    <row r="5" spans="1:6">
+      <c r="A5" s="24">
         <v>45974</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="31">
+    <row r="6" spans="1:6">
+      <c r="A6" s="30">
         <v>45975</v>
       </c>
-      <c r="B6" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="32" t="s">
-        <v>314</v>
-      </c>
-      <c r="D6" s="32" t="s">
-        <v>326</v>
-      </c>
-      <c r="E6" s="32" t="s">
-        <v>376</v>
-      </c>
-      <c r="F6" s="32" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="45" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="33">
+      <c r="B6" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>321</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>371</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="32">
         <v>45987</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="45" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="33">
+    <row r="8" spans="1:6">
+      <c r="A8" s="32">
         <v>45998</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="45" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="46">
+    <row r="9" spans="1:6">
+      <c r="A9" s="38">
         <v>46006</v>
       </c>
-      <c r="B9" s="47" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="47" t="s">
-        <v>405</v>
-      </c>
-      <c r="D9" s="47" t="s">
-        <v>406</v>
-      </c>
-      <c r="E9" s="47" t="s">
-        <v>407</v>
-      </c>
-      <c r="F9" s="47" t="s">
+      <c r="B9" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>400</v>
+      </c>
+      <c r="D9" s="31" t="s">
+        <v>401</v>
+      </c>
+      <c r="E9" s="31" t="s">
+        <v>402</v>
+      </c>
+      <c r="F9" s="31" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:6" s="45" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="33">
+    <row r="10" spans="1:6">
+      <c r="A10" s="32">
         <v>46021</v>
       </c>
-      <c r="B10" s="39" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10" s="39" t="s">
-        <v>405</v>
-      </c>
-      <c r="D10" s="39" t="s">
-        <v>374</v>
-      </c>
-      <c r="E10" s="39" t="s">
-        <v>422</v>
-      </c>
-      <c r="F10" s="39" t="s">
-        <v>67</v>
+      <c r="B10" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>400</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="32">
+        <v>46107</v>
+      </c>
+      <c r="B11" s="55" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="55" t="s">
+        <v>478</v>
+      </c>
+      <c r="D11" s="55" t="s">
+        <v>490</v>
+      </c>
+      <c r="E11" s="51" t="s">
+        <v>491</v>
+      </c>
+      <c r="F11" s="55" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="32">
+        <v>46107</v>
+      </c>
+      <c r="B12" s="55" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="55" t="s">
+        <v>478</v>
+      </c>
+      <c r="D12" s="55" t="s">
+        <v>492</v>
+      </c>
+      <c r="E12" s="51" t="s">
+        <v>493</v>
+      </c>
+      <c r="F12" s="55" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="32">
+        <v>46107</v>
+      </c>
+      <c r="B13" s="55" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="55" t="s">
+        <v>494</v>
+      </c>
+      <c r="D13" s="55" t="s">
+        <v>495</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>496</v>
+      </c>
+      <c r="F13" s="55" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="32">
+        <v>46107</v>
+      </c>
+      <c r="B14" s="55" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="55" t="s">
+        <v>498</v>
+      </c>
+      <c r="D14" s="55" t="s">
+        <v>497</v>
+      </c>
+      <c r="E14" s="51" t="s">
+        <v>499</v>
+      </c>
+      <c r="F14" s="55" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="32">
+        <v>46107</v>
+      </c>
+      <c r="B15" s="55" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="55" t="s">
+        <v>498</v>
+      </c>
+      <c r="D15" s="55" t="s">
+        <v>497</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>500</v>
+      </c>
+      <c r="F15" s="55" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>